<commit_message>
refactor generic plot functions
</commit_message>
<xml_diff>
--- a/docs/downloads/04/tbl_age_obs_alaotra_tous.xlsx
+++ b/docs/downloads/04/tbl_age_obs_alaotra_tous.xlsx
@@ -379,7 +379,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Alaotra - Ambatoharanana</t>
+          <t>Ambatoharanana</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -397,7 +397,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Alaotra - Ambatoharanana</t>
+          <t>Ambatoharanana</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -415,7 +415,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Alaotra - Ambatoharanana</t>
+          <t>Ambatoharanana</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -433,7 +433,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Alaotra - Ambatoharanana</t>
+          <t>Ambatoharanana</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -451,7 +451,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Alaotra - Ambatoharanana</t>
+          <t>Ambatoharanana</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -469,7 +469,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Alaotra - Ambatoharanana</t>
+          <t>Ambatoharanana</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -487,7 +487,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Alaotra - Ambatoharanana</t>
+          <t>Ambatoharanana</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -499,7 +499,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Alaotra - Ambatoharanana</t>
+          <t>Ambatoharanana</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -511,7 +511,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Alaotra - Ambatomanga</t>
+          <t>Ambatomanga</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -529,7 +529,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Alaotra - Ambatomanga</t>
+          <t>Ambatomanga</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -547,7 +547,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Alaotra - Ambatomanga</t>
+          <t>Ambatomanga</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -565,7 +565,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Alaotra - Ambatomanga</t>
+          <t>Ambatomanga</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -583,7 +583,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Alaotra - Ambatomanga</t>
+          <t>Ambatomanga</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -601,7 +601,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Alaotra - Ambatomanga</t>
+          <t>Ambatomanga</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -619,7 +619,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Alaotra - Ambatomanga</t>
+          <t>Ambatomanga</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -637,7 +637,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Alaotra - Ambatomanga</t>
+          <t>Ambatomanga</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -655,7 +655,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Alaotra - Ambodivoara</t>
+          <t>Ambodivoara</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -673,7 +673,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Alaotra - Ambodivoara</t>
+          <t>Ambodivoara</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -691,7 +691,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Alaotra - Ambodivoara</t>
+          <t>Ambodivoara</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -709,7 +709,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Alaotra - Ambodivoara</t>
+          <t>Ambodivoara</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -727,7 +727,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Alaotra - Ambodivoara</t>
+          <t>Ambodivoara</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -745,7 +745,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Alaotra - Ambodivoara</t>
+          <t>Ambodivoara</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -763,7 +763,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Alaotra - Ambodivoara</t>
+          <t>Ambodivoara</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -781,7 +781,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Alaotra - Ambodivoara</t>
+          <t>Ambodivoara</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -793,7 +793,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Alaotra - Ambohidrony</t>
+          <t>Ambohidrony</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -811,7 +811,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Alaotra - Ambohidrony</t>
+          <t>Ambohidrony</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -829,7 +829,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Alaotra - Ambohidrony</t>
+          <t>Ambohidrony</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -847,7 +847,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Alaotra - Ambohidrony</t>
+          <t>Ambohidrony</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -865,7 +865,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Alaotra - Ambohidrony</t>
+          <t>Ambohidrony</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -883,7 +883,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Alaotra - Ambohidrony</t>
+          <t>Ambohidrony</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -901,7 +901,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Alaotra - Ambohidrony</t>
+          <t>Ambohidrony</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -913,7 +913,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Alaotra - Ambohidrony</t>
+          <t>Ambohidrony</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -931,7 +931,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Alaotra - Analamiranga</t>
+          <t>Analamiranga</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -949,7 +949,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Alaotra - Analamiranga</t>
+          <t>Analamiranga</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -967,7 +967,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Alaotra - Analamiranga</t>
+          <t>Analamiranga</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -985,7 +985,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Alaotra - Analamiranga</t>
+          <t>Analamiranga</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1003,7 +1003,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Alaotra - Analamiranga</t>
+          <t>Analamiranga</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1021,7 +1021,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Alaotra - Analamiranga</t>
+          <t>Analamiranga</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1039,7 +1039,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Alaotra - Analamiranga</t>
+          <t>Analamiranga</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1057,7 +1057,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Alaotra - Analamiranga</t>
+          <t>Analamiranga</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1069,7 +1069,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Alaotra - Avaradrano</t>
+          <t>Avaradrano</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1087,7 +1087,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Alaotra - Avaradrano</t>
+          <t>Avaradrano</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1105,7 +1105,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Alaotra - Avaradrano</t>
+          <t>Avaradrano</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1123,7 +1123,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Alaotra - Avaradrano</t>
+          <t>Avaradrano</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1141,7 +1141,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Alaotra - Avaradrano</t>
+          <t>Avaradrano</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1159,7 +1159,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Alaotra - Avaradrano</t>
+          <t>Avaradrano</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1177,7 +1177,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Alaotra - Avaradrano</t>
+          <t>Avaradrano</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1195,7 +1195,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Alaotra - Avaradrano</t>
+          <t>Avaradrano</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1213,7 +1213,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Alaotra - Feramanga Atsimo</t>
+          <t>Feramanga Atsimo</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1231,7 +1231,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Alaotra - Feramanga Atsimo</t>
+          <t>Feramanga Atsimo</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -1249,7 +1249,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Alaotra - Feramanga Atsimo</t>
+          <t>Feramanga Atsimo</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -1267,7 +1267,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Alaotra - Feramanga Atsimo</t>
+          <t>Feramanga Atsimo</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -1285,7 +1285,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Alaotra - Feramanga Atsimo</t>
+          <t>Feramanga Atsimo</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1303,7 +1303,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Alaotra - Feramanga Atsimo</t>
+          <t>Feramanga Atsimo</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -1321,7 +1321,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Alaotra - Feramanga Atsimo</t>
+          <t>Feramanga Atsimo</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -1339,7 +1339,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Alaotra - Feramanga Atsimo</t>
+          <t>Feramanga Atsimo</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -1357,7 +1357,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Alaotra - Mangabe</t>
+          <t>Mangabe</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -1375,7 +1375,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Alaotra - Mangabe</t>
+          <t>Mangabe</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -1393,7 +1393,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Alaotra - Mangabe</t>
+          <t>Mangabe</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -1411,7 +1411,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Alaotra - Mangabe</t>
+          <t>Mangabe</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -1429,7 +1429,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Alaotra - Mangabe</t>
+          <t>Mangabe</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1447,7 +1447,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Alaotra - Mangabe</t>
+          <t>Mangabe</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -1465,7 +1465,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Alaotra - Mangabe</t>
+          <t>Mangabe</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1483,7 +1483,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Alaotra - Mangabe</t>
+          <t>Mangabe</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -1501,7 +1501,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Alaotra - Tous</t>
+          <t>Tous</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -1519,7 +1519,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Alaotra - Tous</t>
+          <t>Tous</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -1537,7 +1537,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Alaotra - Tous</t>
+          <t>Tous</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -1555,7 +1555,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Alaotra - Tous</t>
+          <t>Tous</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -1573,7 +1573,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Alaotra - Tous</t>
+          <t>Tous</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -1591,7 +1591,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Alaotra - Tous</t>
+          <t>Tous</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -1609,7 +1609,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Alaotra - Tous</t>
+          <t>Tous</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -1627,7 +1627,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Alaotra - Tous</t>
+          <t>Tous</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">

</xml_diff>